<commit_message>
Please provide the specific changes or files you would like summarized so I can generate the commit message for you.
</commit_message>
<xml_diff>
--- a/backend/templates/TIR_template.xlsx
+++ b/backend/templates/TIR_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Prodeklarant\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCF1D88-7F87-4F10-A66A-B15CD647D428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CD7D5D-9C30-4AF3-9D65-7B55AF2C518B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -357,31 +357,31 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="4"/>
+    </xf>
+    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="4"/>
-    </xf>
-    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="21">
@@ -895,10 +895,10 @@
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="6"/>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
@@ -920,8 +920,8 @@
     </row>
     <row r="4" spans="1:21">
       <c r="A4" s="6"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
@@ -943,8 +943,8 @@
     </row>
     <row r="5" spans="1:21">
       <c r="A5" s="6"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -1069,9 +1069,9 @@
       <c r="G10" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
-      <c r="J10" s="33"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
       <c r="K10" s="14"/>
       <c r="L10" s="20"/>
       <c r="M10" s="2"/>
@@ -1094,9 +1094,9 @@
       <c r="G11" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="38"/>
       <c r="K11" s="6"/>
       <c r="L11" s="21"/>
       <c r="M11" s="2"/>
@@ -1506,15 +1506,15 @@
       <c r="U29" s="2"/>
     </row>
     <row r="30" spans="2:21">
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
-      <c r="D30" s="38" t="s">
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="E30" s="38"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
       <c r="I30" s="7"/>
       <c r="J30" s="6"/>
       <c r="L30" s="2"/>
@@ -1529,13 +1529,13 @@
       <c r="U30" s="2"/>
     </row>
     <row r="31" spans="2:21">
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="37"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="37"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
       <c r="I31" s="7"/>
       <c r="J31" s="6"/>
       <c r="L31" s="2"/>
@@ -1550,13 +1550,13 @@
       <c r="U31" s="2"/>
     </row>
     <row r="32" spans="2:21">
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="37"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="37"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
       <c r="I32" s="7"/>
       <c r="J32" s="6"/>
       <c r="L32" s="2"/>
@@ -1574,9 +1574,9 @@
       <c r="B33" s="6"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="34"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
       <c r="H33" s="9"/>
       <c r="I33" s="10"/>
       <c r="J33" s="6"/>
@@ -1595,8 +1595,8 @@
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="9"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
       <c r="G34" s="11"/>
       <c r="H34" s="9"/>
       <c r="I34" s="12"/>
@@ -1757,6 +1757,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:H17"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E26:H26"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="E20:H20"/>
     <mergeCell ref="E33:G33"/>
@@ -1773,29 +1796,6 @@
     <mergeCell ref="E27:H27"/>
     <mergeCell ref="E28:H28"/>
     <mergeCell ref="E29:H29"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="E23:H23"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:H17"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.70866141732283472" top="0.62992125984251968" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>